<commit_message>
Fix domain for FA items
</commit_message>
<xml_diff>
--- a/curation/draft/crf/CRF_PR_RS_RadioTherapy.xlsx
+++ b/curation/draft/crf/CRF_PR_RS_RadioTherapy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_github\cdisc-org\COSMoS\curation\draft\crf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECE6D8CF-AE0E-4170-9F8F-F32A6EF2F345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAE5107E-4A8F-4E47-9BAB-3AE0780BAF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="915" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="987" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="987" uniqueCount="240">
   <si>
     <t>This spreadsheet contains CDISC CRF Specializations loaded from 303 YAML files as of 2025-11-26.
 The spreadsheet contains 303 unique CDISC CRF Specializations.
@@ -803,9 +803,6 @@
   </si>
   <si>
     <t>RSDAT</t>
-  </si>
-  <si>
-    <t>FA</t>
   </si>
 </sst>
 </file>
@@ -3129,7 +3126,7 @@
       </c>
       <c r="F18" s="20"/>
       <c r="G18" s="17" t="s">
-        <v>240</v>
+        <v>90</v>
       </c>
       <c r="H18" s="20" t="s">
         <v>223</v>
@@ -3206,7 +3203,7 @@
       </c>
       <c r="F19" s="20"/>
       <c r="G19" s="17" t="s">
-        <v>240</v>
+        <v>90</v>
       </c>
       <c r="H19" s="20" t="s">
         <v>223</v>
@@ -4788,7 +4785,7 @@
       </c>
       <c r="F41" s="20"/>
       <c r="G41" s="17" t="s">
-        <v>240</v>
+        <v>90</v>
       </c>
       <c r="H41" s="20" t="s">
         <v>221</v>
@@ -4865,7 +4862,7 @@
       </c>
       <c r="F42" s="20"/>
       <c r="G42" s="17" t="s">
-        <v>240</v>
+        <v>90</v>
       </c>
       <c r="H42" s="20" t="s">
         <v>221</v>
@@ -5153,12 +5150,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="6f964de0-4574-4146-b206-2188082d0535" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5350,17 +5346,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="6f964de0-4574-4146-b206-2188082d0535" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{754EEFC7-D3AC-4CC2-9E2E-379BA4B1F155}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7F7B728-5317-4606-AFBD-8EBE6F35E39C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6f964de0-4574-4146-b206-2188082d0535"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5384,17 +5389,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7F7B728-5317-4606-AFBD-8EBE6F35E39C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{754EEFC7-D3AC-4CC2-9E2E-379BA4B1F155}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6f964de0-4574-4146-b206-2188082d0535"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>